<commit_message>
n8n board refresh 2026-08-01T17:39:13Z
</commit_message>
<xml_diff>
--- a/app/reports/JTGEY_research.xlsx
+++ b/app/reports/JTGEY_research.xlsx
@@ -614,7 +614,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-07-31 17:38 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
+          <t>Generated 2026-08-01 17:36 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
         </is>
       </c>
     </row>
@@ -851,7 +851,7 @@
         </is>
       </c>
       <c r="B5" s="6" t="n">
-        <v>0.04736999988555908</v>
+        <v>0.04744999885559082</v>
       </c>
     </row>
     <row r="6">

</xml_diff>